<commit_message>
#auto RunMng env snapshot - 2026-04-21 14:36:51
</commit_message>
<xml_diff>
--- a/code/WS_Mdl/Auxi/WB_Diff_NET_sum_Pkg_TEMPLATExlsx.xlsx
+++ b/code/WS_Mdl/Auxi/WB_Diff_NET_sum_Pkg_TEMPLATExlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\code\WS_Mdl\Auxi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC09A356-5DEA-46F5-97C0-916DD6568856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9B0AD06-4B92-4808-9B88-1D059D4BFC3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B600783-26D9-4AA8-9037-2D44D1D76FD3}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4294965429" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4294966225" uniqueCount="33">
   <si>
     <t>Diff</t>
   </si>
@@ -128,10 +128,10 @@
     <t>MdlN_B</t>
   </si>
   <si>
-    <t>%_Pm_S</t>
-  </si>
-  <si>
-    <t>%_Pm_B</t>
+    <t>%_Pm _S</t>
+  </si>
+  <si>
+    <t>%_Pm _B</t>
   </si>
 </sst>
 </file>
@@ -289,18 +289,18 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Mono"/>
       <family val="3"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
       <name val="Aptos Mono"/>
       <family val="3"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Aptos Mono"/>
       <family val="3"/>
     </font>
@@ -726,33 +726,45 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="21" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="21" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="21" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="21" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="21" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1140,368 +1152,368 @@
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
     <col min="2" max="4" width="15.7109375" customWidth="1"/>
     <col min="5" max="7" width="12.7109375" customWidth="1"/>
-    <col min="8" max="8" width="40.7109375" customWidth="1"/>
+    <col min="8" max="8" width="32.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2"/>
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:8" s="27" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="23"/>
+      <c r="B1" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="26" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="14">
+      <c r="B2" s="8">
         <v>64836735</v>
       </c>
-      <c r="C2" s="15">
+      <c r="C2" s="9">
         <v>61860742</v>
       </c>
-      <c r="D2" s="16">
+      <c r="D2" s="10">
         <v>2975993</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="3">
         <v>4.8</v>
       </c>
-      <c r="F2" s="23">
-        <v>9.9</v>
-      </c>
-      <c r="G2" s="23">
-        <v>9.9</v>
-      </c>
-      <c r="H2" s="7" t="s">
+      <c r="F2" s="17">
+        <v>9.9</v>
+      </c>
+      <c r="G2" s="17">
+        <v>9.9</v>
+      </c>
+      <c r="H2" s="20" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="17">
+      <c r="B3" s="11">
         <v>2926633</v>
       </c>
-      <c r="C3" s="18">
+      <c r="C3" s="12">
         <v>2749410</v>
       </c>
-      <c r="D3" s="19">
+      <c r="D3" s="13">
         <v>177223</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="5">
         <v>6.4</v>
       </c>
-      <c r="F3" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="G3" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="H3" s="10" t="s">
+      <c r="F3" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="G3" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="H3" s="21" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="17">
+      <c r="B4" s="11">
         <v>-46991120</v>
       </c>
-      <c r="C4" s="18">
+      <c r="C4" s="12">
         <v>-44566490</v>
       </c>
-      <c r="D4" s="19">
+      <c r="D4" s="13">
         <v>-2424630</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="5">
         <v>5.4</v>
       </c>
-      <c r="F4" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="G4" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="H4" s="10" t="s">
+      <c r="F4" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="G4" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="H4" s="21" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="17">
+      <c r="B5" s="11">
         <v>-361306</v>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="12">
         <v>-3339785</v>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="13">
         <v>2978479</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="5">
         <v>-89.2</v>
       </c>
-      <c r="F5" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="G5" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="H5" s="10" t="s">
+      <c r="F5" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="G5" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="H5" s="21" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="11">
         <v>-1220318</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="12">
         <v>1459169</v>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="13">
         <v>-2679488</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="5">
         <v>-183.6</v>
       </c>
-      <c r="F6" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="G6" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="H6" s="10" t="s">
+      <c r="F6" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="G6" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="H6" s="21" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="20">
+      <c r="B7" s="14">
         <v>-19193189</v>
       </c>
-      <c r="C7" s="21">
+      <c r="C7" s="15">
         <v>-18166141</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="16">
         <v>-1027048</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="7">
         <v>5.7</v>
       </c>
-      <c r="F7" s="25">
-        <v>9.9</v>
-      </c>
-      <c r="G7" s="25">
-        <v>9.9</v>
-      </c>
-      <c r="H7" s="13" t="s">
+      <c r="F7" s="19">
+        <v>9.9</v>
+      </c>
+      <c r="G7" s="19">
+        <v>9.9</v>
+      </c>
+      <c r="H7" s="22" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="8">
         <v>13207082</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="9">
         <v>10797078</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="10">
         <v>2410004</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="3">
         <v>22.3</v>
       </c>
-      <c r="F8" s="23">
-        <v>9.9</v>
-      </c>
-      <c r="G8" s="23">
-        <v>9.9</v>
-      </c>
-      <c r="H8" s="7" t="s">
+      <c r="F8" s="17">
+        <v>9.9</v>
+      </c>
+      <c r="G8" s="17">
+        <v>9.9</v>
+      </c>
+      <c r="H8" s="20" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="11">
         <v>-4427694</v>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="12">
         <v>-4497534</v>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="13">
         <v>69840</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="5">
         <v>-1.6</v>
       </c>
-      <c r="F9" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="G9" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="H9" s="10" t="s">
+      <c r="F9" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="G9" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="H9" s="21" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="17">
+      <c r="B10" s="11">
         <v>-837279</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="12">
         <v>-802160</v>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="13">
         <v>-35119</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="5">
         <v>4.4000000000000004</v>
       </c>
-      <c r="F10" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="G10" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="H10" s="10" t="s">
+      <c r="F10" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="G10" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="H10" s="21" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="11">
         <v>-2814093</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="12">
         <v>-4577399</v>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="13">
         <v>1763306</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="5">
         <v>-38.5</v>
       </c>
-      <c r="F11" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="G11" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="H11" s="10" t="s">
+      <c r="F11" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="G11" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="H11" s="21" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="17">
+      <c r="B12" s="11">
         <v>-2544158</v>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="12">
         <v>-4577399</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="13">
         <v>1763306</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="5">
         <v>-38.5</v>
       </c>
-      <c r="F12" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="G12" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="H12" s="10" t="s">
+      <c r="F12" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="G12" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="H12" s="21" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="17">
+      <c r="B13" s="11">
         <v>5979522</v>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="12">
         <v>7514534</v>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="13">
         <v>-1535012</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="5">
         <v>-20.399999999999999</v>
       </c>
-      <c r="F13" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="G13" s="24">
-        <v>9.9</v>
-      </c>
-      <c r="H13" s="10" t="s">
+      <c r="F13" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="G13" s="18">
+        <v>9.9</v>
+      </c>
+      <c r="H13" s="21" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="20">
+      <c r="B14" s="14">
         <v>-8557153</v>
       </c>
-      <c r="C14" s="21">
+      <c r="C14" s="15">
         <v>-8433782</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="16">
         <v>-123371</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="7">
         <v>1.5</v>
       </c>
-      <c r="F14" s="25">
-        <v>9.9</v>
-      </c>
-      <c r="G14" s="25">
-        <v>9.9</v>
-      </c>
-      <c r="H14" s="13" t="s">
+      <c r="F14" s="19">
+        <v>9.9</v>
+      </c>
+      <c r="G14" s="19">
+        <v>9.9</v>
+      </c>
+      <c r="H14" s="22" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>

<commit_message>
NBr66 ran (fixed Cond regridding)
</commit_message>
<xml_diff>
--- a/code/WS_Mdl/Auxi/WB_Diff_NET_sum_Pkg_TEMPLATExlsx.xlsx
+++ b/code/WS_Mdl/Auxi/WB_Diff_NET_sum_Pkg_TEMPLATExlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\code\WS_Mdl\Auxi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9B0AD06-4B92-4808-9B88-1D059D4BFC3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A46B6E3-3841-43EC-A935-0ADD83387E13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B600783-26D9-4AA8-9037-2D44D1D76FD3}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4294966225" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Diff</t>
   </si>
@@ -128,17 +128,17 @@
     <t>MdlN_B</t>
   </si>
   <si>
-    <t>%_Pm _S</t>
-  </si>
-  <si>
-    <t>%_Pm _B</t>
+    <t>%_Pm_S</t>
+  </si>
+  <si>
+    <t>%_Pm_B</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -299,6 +299,13 @@
       <family val="3"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Aptos Mono"/>
@@ -726,7 +733,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
@@ -751,19 +758,22 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1169,10 +1179,10 @@
       <c r="E1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="G1" s="28" t="s">
         <v>32</v>
       </c>
       <c r="H1" s="26" t="s">

</xml_diff>

<commit_message>
NBr70 finished + added date to WB_Diff
</commit_message>
<xml_diff>
--- a/code/WS_Mdl/Auxi/WB_Diff_NET_sum_Pkg_TEMPLATExlsx.xlsx
+++ b/code/WS_Mdl/Auxi/WB_Diff_NET_sum_Pkg_TEMPLATExlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\code\WS_Mdl\Auxi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A46B6E3-3841-43EC-A935-0ADD83387E13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64BA31DC-11ED-48FD-BABA-11E825695658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B600783-26D9-4AA8-9037-2D44D1D76FD3}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4294966722" uniqueCount="33">
   <si>
     <t>Diff</t>
   </si>
@@ -757,9 +757,6 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -773,6 +770,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1165,27 +1165,27 @@
     <col min="8" max="8" width="32.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="27" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23"/>
-      <c r="B1" s="24" t="s">
+    <row r="1" spans="1:8" s="26" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="28"/>
+      <c r="B1" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="28" t="s">
+      <c r="F1" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="28" t="s">
+      <c r="G1" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="26" t="s">
+      <c r="H1" s="25" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
NBr103 PoP: added SFR_CBC_Par_to_TIF + cleaned up a bit
</commit_message>
<xml_diff>
--- a/code/WS_Mdl/Auxi/WB_Diff_NET_sum_Pkg_TEMPLATExlsx.xlsx
+++ b/code/WS_Mdl/Auxi/WB_Diff_NET_sum_Pkg_TEMPLATExlsx.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\code\WS_Mdl\Auxi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{701B4D8F-4F47-4333-85BC-4347B51541B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69734AE8-C081-438F-B06F-A21C275177A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{0B600783-26D9-4AA8-9037-2D44D1D76FD3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B600783-26D9-4AA8-9037-2D44D1D76FD3}"/>
   </bookViews>
   <sheets>
     <sheet name="Diff" sheetId="1" r:id="rId1"/>
@@ -496,7 +496,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -612,63 +612,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="medium">
         <color indexed="64"/>
       </right>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -683,6 +632,98 @@
     <border>
       <left/>
       <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="double">
         <color indexed="64"/>
       </right>
       <top/>
@@ -736,49 +777,43 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="20" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="20" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="21" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="20" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="20" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="20" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="21" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="21" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1166,361 +1201,361 @@
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
     <col min="2" max="3" width="18.7109375" customWidth="1"/>
     <col min="4" max="4" width="15.7109375" customWidth="1"/>
-    <col min="5" max="7" width="9.7109375" style="26" customWidth="1"/>
+    <col min="5" max="7" width="9.7109375" style="11" customWidth="1"/>
     <col min="8" max="8" width="33.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="20" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="21"/>
-      <c r="B1" s="17" t="s">
+    <row r="1" spans="1:8" s="8" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="22"/>
+      <c r="B1" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="E1" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="22" t="s">
+      <c r="G1" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="H1" s="16" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="2">
         <v>199826958.86136511</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="2">
         <v>199826958.86136511</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="3">
         <v>0</v>
       </c>
-      <c r="E2" s="23">
+      <c r="E2" s="9">
         <v>0</v>
       </c>
-      <c r="F2" s="27">
+      <c r="F2" s="12">
         <v>100</v>
       </c>
-      <c r="G2" s="27">
+      <c r="G2" s="12">
         <v>100</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="H2" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="2">
         <v>3606186.8910699999</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="2">
         <v>3601395.9391399999</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="3">
         <v>4790.9519299995154</v>
       </c>
-      <c r="E3" s="24">
+      <c r="E3" s="9">
         <v>0.13303041406615171</v>
       </c>
-      <c r="F3" s="28">
+      <c r="F3" s="12">
         <v>1.804654843179534</v>
       </c>
-      <c r="G3" s="28">
+      <c r="G3" s="12">
         <v>1.8022572928403311</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="2">
         <v>-111342503.2947228</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="2">
         <v>-111381850.6142258</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="3">
         <v>39347.319503054023</v>
       </c>
-      <c r="E4" s="24">
+      <c r="E4" s="9">
         <v>-3.5326509019260759E-2</v>
       </c>
-      <c r="F4" s="28">
+      <c r="F4" s="12">
         <v>-55.719460441756198</v>
       </c>
-      <c r="G4" s="28">
+      <c r="G4" s="12">
         <v>-55.739151138010222</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="2">
         <v>-13772656.78056813</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="2">
         <v>-13925120.04151663</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="3">
         <v>152463.26094849969</v>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="9">
         <v>-1.0948793295421699</v>
       </c>
-      <c r="F5" s="28">
+      <c r="F5" s="12">
         <v>-6.8922916402502299</v>
       </c>
-      <c r="G5" s="28">
+      <c r="G5" s="12">
         <v>-6.9685892838801244</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="H5" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="2">
         <v>-11475957.0153889</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="2">
         <v>-11594544.07280116</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="3">
         <v>118587.05741225369</v>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="9">
         <v>-1.0227832734746241</v>
       </c>
-      <c r="F6" s="28">
+      <c r="F6" s="12">
         <v>-5.7429473384272614</v>
       </c>
-      <c r="G6" s="28">
+      <c r="G6" s="12">
         <v>-5.8022922126564316</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="H6" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="17">
         <v>-66805023.657589316</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="17">
         <v>-66573010.299593009</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="18">
         <v>-232013.35799630731</v>
       </c>
-      <c r="E7" s="25">
+      <c r="E7" s="19">
         <v>0.34850963919491817</v>
       </c>
-      <c r="F7" s="29">
+      <c r="F7" s="20">
         <v>-33.431436898330112</v>
       </c>
-      <c r="G7" s="29">
+      <c r="G7" s="20">
         <v>-33.315329762777253</v>
       </c>
-      <c r="H7" s="16" t="s">
+      <c r="H7" s="21" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="2">
         <v>64163384</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="2">
         <v>63878528</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="3">
         <v>284856</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="9">
         <v>0.44593388250900212</v>
       </c>
-      <c r="F8" s="27">
+      <c r="F8" s="12">
         <v>32.109473299103222</v>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="12">
         <v>31.966921962875549</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="2">
         <v>-11076712</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="2">
         <v>-11353562</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="3">
         <v>276850</v>
       </c>
-      <c r="E9" s="24">
+      <c r="E9" s="9">
         <v>-2.438441785934669</v>
       </c>
-      <c r="F9" s="28">
+      <c r="F9" s="12">
         <v>-5.5431519666396687</v>
       </c>
-      <c r="G9" s="28">
+      <c r="G9" s="12">
         <v>-5.6816968364497882</v>
       </c>
-      <c r="H9" s="15" t="s">
+      <c r="H9" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="2">
         <v>-11507343</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="2">
         <v>-11692030</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="3">
         <v>184687</v>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="9">
         <v>-1.579597383858919</v>
       </c>
-      <c r="F10" s="28">
+      <c r="F10" s="12">
         <v>-5.7586539201567426</v>
       </c>
-      <c r="G10" s="28">
+      <c r="G10" s="12">
         <v>-5.8510773854651097</v>
       </c>
-      <c r="H10" s="15" t="s">
+      <c r="H10" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="2">
         <v>-21015166</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="2">
         <v>-30031516</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="3">
         <v>9016350</v>
       </c>
-      <c r="E11" s="24">
+      <c r="E11" s="9">
         <v>-30.022959879880851</v>
       </c>
-      <c r="F11" s="28">
+      <c r="F11" s="12">
         <v>-10.516682093220361</v>
       </c>
-      <c r="G11" s="28">
+      <c r="G11" s="12">
         <v>-15.02876096955222</v>
       </c>
-      <c r="H11" s="15" t="s">
+      <c r="H11" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="2">
         <v>-9739188</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="28">
+      <c r="C12" s="2"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="12">
         <v>-4.8738108488939194</v>
       </c>
-      <c r="G12" s="28"/>
-      <c r="H12" s="15" t="s">
+      <c r="G12" s="12"/>
+      <c r="H12" s="6" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="2">
         <v>2306720</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="2">
         <v>2267144</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="3">
         <v>39576</v>
       </c>
-      <c r="E13" s="24">
+      <c r="E13" s="9">
         <v>1.7456323903554429</v>
       </c>
-      <c r="F13" s="28">
+      <c r="F13" s="12">
         <v>1.1543587577691881</v>
       </c>
-      <c r="G13" s="28">
+      <c r="G13" s="12">
         <v>1.1345536222531849</v>
       </c>
-      <c r="H13" s="15" t="s">
+      <c r="H13" s="6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="4">
         <v>-13039333</v>
       </c>
-      <c r="C14" s="12">
+      <c r="C14" s="4">
         <v>-13035376</v>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="5">
         <v>-3957</v>
       </c>
-      <c r="E14" s="25">
+      <c r="E14" s="10">
         <v>3.035585624841201E-2</v>
       </c>
-      <c r="F14" s="29">
+      <c r="F14" s="13">
         <v>-6.5253122372974524</v>
       </c>
-      <c r="G14" s="29">
+      <c r="G14" s="13">
         <v>-6.5233320240056374</v>
       </c>
-      <c r="H14" s="16" t="s">
+      <c r="H14" s="7" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>